<commit_message>
created Rmarkdown file for appendix and made some changes to the variable names in ISIC graph/tables
</commit_message>
<xml_diff>
--- a/Peter/Sectoral Analysis (ISIC)/ISIC3/ISIC3 Jamacia average.xlsx
+++ b/Peter/Sectoral Analysis (ISIC)/ISIC3/ISIC3 Jamacia average.xlsx
@@ -1,61 +1,68 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Bede7/Desktop/RA/rproj-NatlAccountsSectorData/Peter/Sectoral Analysis (ISIC)/ISIC3/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7FDFFB-66DE-1345-978E-55DCFAED9632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="20620" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t xml:space="preserve">Primary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manufacturing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electricity, gas, water supply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Construction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transportation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotels and restaurants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Communications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financial Intermediation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real Estate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other: commercial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other: public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sum</t>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Electricity, gas, water supply</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
+    <t>Transportation</t>
+  </si>
+  <si>
+    <t>Communications</t>
+  </si>
+  <si>
+    <t>Financial Intermediation</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Other: commercial</t>
+  </si>
+  <si>
+    <t>Other: public</t>
+  </si>
+  <si>
+    <t>sum</t>
+  </si>
+  <si>
+    <t>Hospitality</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -91,6 +98,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -372,11 +388,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -393,67 +409,67 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>0.0819980599389136</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0837615443201281</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.0307194920807062</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.0707464652977753</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.0617295374349217</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.0701289888106766</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.0226769755394498</v>
-      </c>
-      <c r="H2" t="n">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>8.1998059938913598E-2</v>
+      </c>
+      <c r="B2">
+        <v>8.3761544320128098E-2</v>
+      </c>
+      <c r="C2">
+        <v>3.07194920807062E-2</v>
+      </c>
+      <c r="D2">
+        <v>7.0746465297775299E-2</v>
+      </c>
+      <c r="E2">
+        <v>6.1729537434921697E-2</v>
+      </c>
+      <c r="F2">
+        <v>7.0128988810676599E-2</v>
+      </c>
+      <c r="G2">
+        <v>2.2676975539449799E-2</v>
+      </c>
+      <c r="H2">
         <v>0.104525146280328</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>0.102503377600836</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>0.191604766182386</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2">
         <v>0.179605646513881</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding ISIC 3 to appendix
</commit_message>
<xml_diff>
--- a/Peter/Sectoral Analysis (ISIC)/ISIC3/ISIC3 Jamacia average.xlsx
+++ b/Peter/Sectoral Analysis (ISIC)/ISIC3/ISIC3 Jamacia average.xlsx
@@ -1,68 +1,61 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Bede7/Desktop/RA/rproj-NatlAccountsSectorData/Peter/Sectoral Analysis (ISIC)/ISIC3/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7FDFFB-66DE-1345-978E-55DCFAED9632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="20620" windowHeight="13660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Manufacturing</t>
-  </si>
-  <si>
-    <t>Electricity, gas, water supply</t>
-  </si>
-  <si>
-    <t>Construction</t>
-  </si>
-  <si>
-    <t>Transportation</t>
-  </si>
-  <si>
-    <t>Communications</t>
-  </si>
-  <si>
-    <t>Financial Intermediation</t>
-  </si>
-  <si>
-    <t>Real Estate</t>
-  </si>
-  <si>
-    <t>Other: commercial</t>
-  </si>
-  <si>
-    <t>Other: public</t>
-  </si>
-  <si>
-    <t>sum</t>
-  </si>
-  <si>
-    <t>Hospitality</t>
+    <t xml:space="preserve">Primary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity, gas, water supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transportation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospitality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Communications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financial Intermediation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real Estate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other: Private</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other: Public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sum</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -98,15 +91,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -388,11 +372,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -409,67 +393,67 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>8.1998059938913598E-2</v>
-      </c>
-      <c r="B2">
-        <v>8.3761544320128098E-2</v>
-      </c>
-      <c r="C2">
-        <v>3.07194920807062E-2</v>
-      </c>
-      <c r="D2">
-        <v>7.0746465297775299E-2</v>
-      </c>
-      <c r="E2">
-        <v>6.1729537434921697E-2</v>
-      </c>
-      <c r="F2">
-        <v>7.0128988810676599E-2</v>
-      </c>
-      <c r="G2">
-        <v>2.2676975539449799E-2</v>
-      </c>
-      <c r="H2">
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0.0819980599389136</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.083761544320128</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0307194920807062</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0707464652977752</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0617295374349217</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0701289888106766</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0226769755394498</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.104525146280328</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>0.102503377600836</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="n">
         <v>0.191604766182386</v>
       </c>
-      <c r="K2">
+      <c r="K2" t="n">
         <v>0.179605646513881</v>
       </c>
-      <c r="L2">
+      <c r="L2" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>